<commit_message>
feat(users): enhance user retrieval by allowing Super Admin to specify organization or retrieve all users
</commit_message>
<xml_diff>
--- a/convert-to-excel/assets_demo.xlsx
+++ b/convert-to-excel/assets_demo.xlsx
@@ -397,29 +397,47 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:M6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>assetName</v>
+        <v>Name</v>
       </c>
       <c r="B1" t="str">
-        <v>category</v>
+        <v>Asset Tag</v>
       </c>
       <c r="C1" t="str">
-        <v>assetType</v>
+        <v>Type</v>
       </c>
       <c r="D1" t="str">
-        <v>model</v>
+        <v>Category</v>
       </c>
       <c r="E1" t="str">
-        <v>location</v>
+        <v>Location</v>
       </c>
       <c r="F1" t="str">
-        <v>purchaseDate</v>
+        <v>Manufacturer</v>
       </c>
       <c r="G1" t="str">
-        <v>value</v>
+        <v>Model</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Serial Number</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Purchase Date</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Purchase Cost</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Warranty Expiry</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Description</v>
       </c>
     </row>
     <row r="2">
@@ -427,22 +445,40 @@
         <v>Central Air Conditioning Unit</v>
       </c>
       <c r="B2" t="str">
+        <v>AST-HVAC-001</v>
+      </c>
+      <c r="C2" t="str">
+        <v>immovable</v>
+      </c>
+      <c r="D2" t="str">
         <v>HVAC</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Movable</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Daikin VRV IV</v>
       </c>
       <c r="E2" t="str">
         <v>Building A - Roof</v>
       </c>
       <c r="F2" t="str">
+        <v>Daikin</v>
+      </c>
+      <c r="G2" t="str">
+        <v>VRV IV</v>
+      </c>
+      <c r="H2" t="str">
+        <v>DK-99231</v>
+      </c>
+      <c r="I2" t="str">
         <v>2023-06-12</v>
       </c>
-      <c r="G2">
+      <c r="J2" t="str">
         <v>8500</v>
+      </c>
+      <c r="K2" t="str">
+        <v>2028-06-12</v>
+      </c>
+      <c r="L2" t="str">
+        <v>active</v>
+      </c>
+      <c r="M2" t="str">
+        <v>Primary AC unit for Building A</v>
       </c>
     </row>
     <row r="3">
@@ -450,22 +486,40 @@
         <v>Water Pump System</v>
       </c>
       <c r="B3" t="str">
+        <v>AST-PLUMB-002</v>
+      </c>
+      <c r="C3" t="str">
+        <v>movable</v>
+      </c>
+      <c r="D3" t="str">
         <v>Plumbing</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Movable</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Grundfos CRN10</v>
       </c>
       <c r="E3" t="str">
         <v>Basement Pump Room</v>
       </c>
       <c r="F3" t="str">
+        <v>Grundfos</v>
+      </c>
+      <c r="G3" t="str">
+        <v>CRN10</v>
+      </c>
+      <c r="H3" t="str">
+        <v>GR-11203</v>
+      </c>
+      <c r="I3" t="str">
         <v>2022-03-08</v>
       </c>
-      <c r="G3">
+      <c r="J3" t="str">
         <v>3200</v>
+      </c>
+      <c r="K3" t="str">
+        <v>2025-03-08</v>
+      </c>
+      <c r="L3" t="str">
+        <v>active</v>
+      </c>
+      <c r="M3" t="str">
+        <v>Main water supply pump</v>
       </c>
     </row>
     <row r="4">
@@ -473,22 +527,40 @@
         <v>Main Power Distribution Panel</v>
       </c>
       <c r="B4" t="str">
+        <v>AST-ELEC-003</v>
+      </c>
+      <c r="C4" t="str">
+        <v>immovable</v>
+      </c>
+      <c r="D4" t="str">
         <v>Electrical</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Immovable</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Schneider Electric Panel</v>
       </c>
       <c r="E4" t="str">
         <v>Electrical Room - Floor 1</v>
       </c>
       <c r="F4" t="str">
+        <v>Schneider Electric</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Square D</v>
+      </c>
+      <c r="H4" t="str">
+        <v>SE-55410</v>
+      </c>
+      <c r="I4" t="str">
         <v>2021-11-20</v>
       </c>
-      <c r="G4">
+      <c r="J4" t="str">
         <v>6400</v>
+      </c>
+      <c r="K4" t="str">
+        <v>2031-11-20</v>
+      </c>
+      <c r="L4" t="str">
+        <v>active</v>
+      </c>
+      <c r="M4" t="str">
+        <v>Primary electrical panel for Floor 1</v>
       </c>
     </row>
     <row r="5">
@@ -496,22 +568,40 @@
         <v>CNC Milling Machine</v>
       </c>
       <c r="B5" t="str">
+        <v>AST-MACH-004</v>
+      </c>
+      <c r="C5" t="str">
+        <v>movable</v>
+      </c>
+      <c r="D5" t="str">
         <v>Machinery</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Movable</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Haas VF-2</v>
       </c>
       <c r="E5" t="str">
         <v>Production Floor</v>
       </c>
       <c r="F5" t="str">
+        <v>Haas</v>
+      </c>
+      <c r="G5" t="str">
+        <v>VF-2</v>
+      </c>
+      <c r="H5" t="str">
+        <v>H-123445</v>
+      </c>
+      <c r="I5" t="str">
         <v>2020-09-14</v>
       </c>
-      <c r="G5">
+      <c r="J5" t="str">
         <v>45000</v>
+      </c>
+      <c r="K5" t="str">
+        <v>2025-09-14</v>
+      </c>
+      <c r="L5" t="str">
+        <v>maintenance</v>
+      </c>
+      <c r="M5" t="str">
+        <v>Precision milling machine</v>
       </c>
     </row>
     <row r="6">
@@ -519,27 +609,45 @@
         <v>Company Delivery Van</v>
       </c>
       <c r="B6" t="str">
+        <v>AST-VEH-005</v>
+      </c>
+      <c r="C6" t="str">
+        <v>movable</v>
+      </c>
+      <c r="D6" t="str">
         <v>Vehicles</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Movable</v>
-      </c>
-      <c r="D6" t="str">
-        <v>Ford Transit 2022</v>
       </c>
       <c r="E6" t="str">
         <v>Parking Lot B</v>
       </c>
       <c r="F6" t="str">
+        <v>Ford</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Transit 2022</v>
+      </c>
+      <c r="H6" t="str">
+        <v>VIN-192837465</v>
+      </c>
+      <c r="I6" t="str">
         <v>2022-01-18</v>
       </c>
-      <c r="G6">
+      <c r="J6" t="str">
         <v>38000</v>
+      </c>
+      <c r="K6" t="str">
+        <v>2027-01-18</v>
+      </c>
+      <c r="L6" t="str">
+        <v>active</v>
+      </c>
+      <c r="M6" t="str">
+        <v>Fleet delivery vehicle</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: Update sample asset and inventory data and regenerate corresponding demo Excel files.
</commit_message>
<xml_diff>
--- a/convert-to-excel/assets_demo.xlsx
+++ b/convert-to-excel/assets_demo.xlsx
@@ -442,207 +442,207 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Central Air Conditioning Unit</v>
+        <v>Precision Lathe X-100</v>
       </c>
       <c r="B2" t="str">
-        <v>AST-HVAC-001</v>
+        <v>AST-MACH-010</v>
       </c>
       <c r="C2" t="str">
-        <v>immovable</v>
+        <v>movable</v>
       </c>
       <c r="D2" t="str">
-        <v>HVAC</v>
+        <v>Machinery</v>
       </c>
       <c r="E2" t="str">
-        <v>Building A - Roof</v>
+        <v>Workshop Floor 1</v>
       </c>
       <c r="F2" t="str">
-        <v>Daikin</v>
+        <v>Mazak</v>
       </c>
       <c r="G2" t="str">
-        <v>VRV IV</v>
+        <v>Quick Turn 100</v>
       </c>
       <c r="H2" t="str">
-        <v>DK-99231</v>
+        <v>MZ-100293</v>
       </c>
       <c r="I2" t="str">
-        <v>2023-06-12</v>
+        <v>2024-01-15</v>
       </c>
       <c r="J2" t="str">
-        <v>8500</v>
+        <v>125000</v>
       </c>
       <c r="K2" t="str">
-        <v>2028-06-12</v>
+        <v>2027-01-15</v>
       </c>
       <c r="L2" t="str">
         <v>active</v>
       </c>
       <c r="M2" t="str">
-        <v>Primary AC unit for Building A</v>
+        <v>High-precision lathe for metalworking</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Water Pump System</v>
+        <v>Server Rack Alpha</v>
       </c>
       <c r="B3" t="str">
-        <v>AST-PLUMB-002</v>
+        <v>AST-IT-020</v>
       </c>
       <c r="C3" t="str">
-        <v>movable</v>
+        <v>immovable</v>
       </c>
       <c r="D3" t="str">
-        <v>Plumbing</v>
+        <v>IT Infrastructure</v>
       </c>
       <c r="E3" t="str">
-        <v>Basement Pump Room</v>
+        <v>Data Center Room 4</v>
       </c>
       <c r="F3" t="str">
-        <v>Grundfos</v>
+        <v>Dell</v>
       </c>
       <c r="G3" t="str">
-        <v>CRN10</v>
+        <v>PowerEdge R750</v>
       </c>
       <c r="H3" t="str">
-        <v>GR-11203</v>
+        <v>DL-SERV-7501</v>
       </c>
       <c r="I3" t="str">
-        <v>2022-03-08</v>
+        <v>2023-11-10</v>
       </c>
       <c r="J3" t="str">
-        <v>3200</v>
+        <v>12000</v>
       </c>
       <c r="K3" t="str">
-        <v>2025-03-08</v>
+        <v>2026-11-10</v>
       </c>
       <c r="L3" t="str">
         <v>active</v>
       </c>
       <c r="M3" t="str">
-        <v>Main water supply pump</v>
+        <v>Primary database server rack</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Main Power Distribution Panel</v>
+        <v>Electric Forklift</v>
       </c>
       <c r="B4" t="str">
-        <v>AST-ELEC-003</v>
+        <v>AST-LOG-030</v>
       </c>
       <c r="C4" t="str">
-        <v>immovable</v>
+        <v>movable</v>
       </c>
       <c r="D4" t="str">
-        <v>Electrical</v>
+        <v>Logistics</v>
       </c>
       <c r="E4" t="str">
-        <v>Electrical Room - Floor 1</v>
+        <v>Warehouse Loading Dock</v>
       </c>
       <c r="F4" t="str">
-        <v>Schneider Electric</v>
+        <v>Toyota</v>
       </c>
       <c r="G4" t="str">
-        <v>Square D</v>
+        <v>8FBMT25</v>
       </c>
       <c r="H4" t="str">
-        <v>SE-55410</v>
+        <v>TY-FL-9912</v>
       </c>
       <c r="I4" t="str">
-        <v>2021-11-20</v>
+        <v>2023-05-20</v>
       </c>
       <c r="J4" t="str">
-        <v>6400</v>
+        <v>45000</v>
       </c>
       <c r="K4" t="str">
-        <v>2031-11-20</v>
+        <v>2026-05-20</v>
       </c>
       <c r="L4" t="str">
         <v>active</v>
       </c>
       <c r="M4" t="str">
-        <v>Primary electrical panel for Floor 1</v>
+        <v>Electric counterbalanced forklift</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>CNC Milling Machine</v>
+        <v>Backup Generator 500kW</v>
       </c>
       <c r="B5" t="str">
-        <v>AST-MACH-004</v>
+        <v>AST-UTIL-040</v>
       </c>
       <c r="C5" t="str">
-        <v>movable</v>
+        <v>immovable</v>
       </c>
       <c r="D5" t="str">
-        <v>Machinery</v>
+        <v>Utilities</v>
       </c>
       <c r="E5" t="str">
-        <v>Production Floor</v>
+        <v>Exterior - North Side</v>
       </c>
       <c r="F5" t="str">
-        <v>Haas</v>
+        <v>Cummins</v>
       </c>
       <c r="G5" t="str">
-        <v>VF-2</v>
+        <v>C500D5P</v>
       </c>
       <c r="H5" t="str">
-        <v>H-123445</v>
+        <v>CM-GEN-500K</v>
       </c>
       <c r="I5" t="str">
-        <v>2020-09-14</v>
+        <v>2022-08-05</v>
       </c>
       <c r="J5" t="str">
-        <v>45000</v>
+        <v>75000</v>
       </c>
       <c r="K5" t="str">
-        <v>2025-09-14</v>
+        <v>2027-08-05</v>
       </c>
       <c r="L5" t="str">
-        <v>maintenance</v>
+        <v>active</v>
       </c>
       <c r="M5" t="str">
-        <v>Precision milling machine</v>
+        <v>Emergency backup power system</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Company Delivery Van</v>
+        <v>Industrial 3D Printer</v>
       </c>
       <c r="B6" t="str">
-        <v>AST-VEH-005</v>
+        <v>AST-RND-050</v>
       </c>
       <c r="C6" t="str">
         <v>movable</v>
       </c>
       <c r="D6" t="str">
-        <v>Vehicles</v>
+        <v>Research &amp; Development</v>
       </c>
       <c r="E6" t="str">
-        <v>Parking Lot B</v>
+        <v>Lab Room 2</v>
       </c>
       <c r="F6" t="str">
-        <v>Ford</v>
+        <v>Stratasys</v>
       </c>
       <c r="G6" t="str">
-        <v>Transit 2022</v>
+        <v>F370</v>
       </c>
       <c r="H6" t="str">
-        <v>VIN-192837465</v>
+        <v>SS-3DP-7482</v>
       </c>
       <c r="I6" t="str">
-        <v>2022-01-18</v>
+        <v>2024-02-12</v>
       </c>
       <c r="J6" t="str">
-        <v>38000</v>
+        <v>55000</v>
       </c>
       <c r="K6" t="str">
-        <v>2027-01-18</v>
+        <v>2026-02-12</v>
       </c>
       <c r="L6" t="str">
         <v>active</v>
       </c>
       <c r="M6" t="str">
-        <v>Fleet delivery vehicle</v>
+        <v>FDM 3D printer for prototyping</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Implement comprehensive inventory management with API, services, and dedicated frontend pages.
</commit_message>
<xml_diff>
--- a/convert-to-excel/assets_demo.xlsx
+++ b/convert-to-excel/assets_demo.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:M16"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -645,9 +645,419 @@
         <v>FDM 3D printer for prototyping</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Central AC Chiller</v>
+      </c>
+      <c r="B7" t="str">
+        <v>AST-HVAC-060</v>
+      </c>
+      <c r="C7" t="str">
+        <v>immovable</v>
+      </c>
+      <c r="D7" t="str">
+        <v>HVAC</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Rooftop - Block A</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Carrier</v>
+      </c>
+      <c r="G7" t="str">
+        <v>AquaEdge 19XR</v>
+      </c>
+      <c r="H7" t="str">
+        <v>CR-HVAC-9002</v>
+      </c>
+      <c r="I7" t="str">
+        <v>2023-03-12</v>
+      </c>
+      <c r="J7" t="str">
+        <v>185000</v>
+      </c>
+      <c r="K7" t="str">
+        <v>2028-03-12</v>
+      </c>
+      <c r="L7" t="str">
+        <v>active</v>
+      </c>
+      <c r="M7" t="str">
+        <v>Main centrifugal chiller for office cooling</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>CCTV Control Hub</v>
+      </c>
+      <c r="B8" t="str">
+        <v>AST-SEC-070</v>
+      </c>
+      <c r="C8" t="str">
+        <v>movable</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Security</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Security Control Room</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Hikvision</v>
+      </c>
+      <c r="G8" t="str">
+        <v>DS-9664NI-I8</v>
+      </c>
+      <c r="H8" t="str">
+        <v>HK-NVR-5542</v>
+      </c>
+      <c r="I8" t="str">
+        <v>2023-09-25</v>
+      </c>
+      <c r="J8" t="str">
+        <v>3500</v>
+      </c>
+      <c r="K8" t="str">
+        <v>2025-09-25</v>
+      </c>
+      <c r="L8" t="str">
+        <v>active</v>
+      </c>
+      <c r="M8" t="str">
+        <v>64-channel network video recorder</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Smart Board Pro 85</v>
+      </c>
+      <c r="B9" t="str">
+        <v>AST-OFF-080</v>
+      </c>
+      <c r="C9" t="str">
+        <v>movable</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Office Equipment</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Conference Room 1</v>
+      </c>
+      <c r="F9" t="str">
+        <v>SMART Technologies</v>
+      </c>
+      <c r="G9" t="str">
+        <v>SBID-7286R</v>
+      </c>
+      <c r="H9" t="str">
+        <v>ST-SB-8501</v>
+      </c>
+      <c r="I9" t="str">
+        <v>2024-01-05</v>
+      </c>
+      <c r="J9" t="str">
+        <v>8500</v>
+      </c>
+      <c r="K9" t="str">
+        <v>2026-01-05</v>
+      </c>
+      <c r="L9" t="str">
+        <v>active</v>
+      </c>
+      <c r="M9" t="str">
+        <v>85-inch interactive 4K display</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Water Filtration System</v>
+      </c>
+      <c r="B10" t="str">
+        <v>AST-UTIL-090</v>
+      </c>
+      <c r="C10" t="str">
+        <v>immovable</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Utilities</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Cafeteria - Back Area</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Kent</v>
+      </c>
+      <c r="G10" t="str">
+        <v>Elite II</v>
+      </c>
+      <c r="H10" t="str">
+        <v>KT-RO-4421</v>
+      </c>
+      <c r="I10" t="str">
+        <v>2023-06-18</v>
+      </c>
+      <c r="J10" t="str">
+        <v>1200</v>
+      </c>
+      <c r="K10" t="str">
+        <v>2024-06-18</v>
+      </c>
+      <c r="L10" t="str">
+        <v>active</v>
+      </c>
+      <c r="M10" t="str">
+        <v>Commercial RO water purification system</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Heavy Duty Air Compressor</v>
+      </c>
+      <c r="B11" t="str">
+        <v>AST-MACH-100</v>
+      </c>
+      <c r="C11" t="str">
+        <v>movable</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Machinery</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Workshop Floor 2</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Ingersoll Rand</v>
+      </c>
+      <c r="G11" t="str">
+        <v>SS3L3</v>
+      </c>
+      <c r="H11" t="str">
+        <v>IR-AC-1092</v>
+      </c>
+      <c r="I11" t="str">
+        <v>2023-12-02</v>
+      </c>
+      <c r="J11" t="str">
+        <v>2800</v>
+      </c>
+      <c r="K11" t="str">
+        <v>2025-12-02</v>
+      </c>
+      <c r="L11" t="str">
+        <v>active</v>
+      </c>
+      <c r="M11" t="str">
+        <v>3HP industrial air compressor</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Hydraulic Power Unit</v>
+      </c>
+      <c r="B12" t="str">
+        <v>AST-MACH-110</v>
+      </c>
+      <c r="C12" t="str">
+        <v>movable</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Machinery</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Workshop Floor 1</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Parker</v>
+      </c>
+      <c r="G12" t="str">
+        <v>HPU-500</v>
+      </c>
+      <c r="H12" t="str">
+        <v>PK-HPU-1122</v>
+      </c>
+      <c r="I12" t="str">
+        <v>2024-03-01</v>
+      </c>
+      <c r="J12" t="str">
+        <v>15000</v>
+      </c>
+      <c r="K12" t="str">
+        <v>2026-03-01</v>
+      </c>
+      <c r="L12" t="str">
+        <v>active</v>
+      </c>
+      <c r="M12" t="str">
+        <v>Heavy-duty hydraulic power supply</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Electric Pallet Jack</v>
+      </c>
+      <c r="B13" t="str">
+        <v>AST-LOG-120</v>
+      </c>
+      <c r="C13" t="str">
+        <v>movable</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Logistics</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Warehouse A</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Raymond</v>
+      </c>
+      <c r="G13" t="str">
+        <v>8210</v>
+      </c>
+      <c r="H13" t="str">
+        <v>RY-PJ-2233</v>
+      </c>
+      <c r="I13" t="str">
+        <v>2023-08-15</v>
+      </c>
+      <c r="J13" t="str">
+        <v>6500</v>
+      </c>
+      <c r="K13" t="str">
+        <v>2025-08-15</v>
+      </c>
+      <c r="L13" t="str">
+        <v>active</v>
+      </c>
+      <c r="M13" t="str">
+        <v>2ton electric walkie pallet jack</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Industrial Exhaust Fan</v>
+      </c>
+      <c r="B14" t="str">
+        <v>AST-HVAC-130</v>
+      </c>
+      <c r="C14" t="str">
+        <v>immovable</v>
+      </c>
+      <c r="D14" t="str">
+        <v>HVAC</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Workshop Ceiling</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Greenheck</v>
+      </c>
+      <c r="G14" t="str">
+        <v>GB-240</v>
+      </c>
+      <c r="H14" t="str">
+        <v>GH-FAN-3344</v>
+      </c>
+      <c r="I14" t="str">
+        <v>2023-10-20</v>
+      </c>
+      <c r="J14" t="str">
+        <v>3200</v>
+      </c>
+      <c r="K14" t="str">
+        <v>2025-10-20</v>
+      </c>
+      <c r="L14" t="str">
+        <v>active</v>
+      </c>
+      <c r="M14" t="str">
+        <v>High-volume exhaust fan for ventilation</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Conveyor Belt System - Section A</v>
+      </c>
+      <c r="B15" t="str">
+        <v>AST-LOG-140</v>
+      </c>
+      <c r="C15" t="str">
+        <v>immovable</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Logistics</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Assembly Line 1</v>
+      </c>
+      <c r="F15" t="str">
+        <v>Hytrol</v>
+      </c>
+      <c r="G15" t="str">
+        <v>TH-50</v>
+      </c>
+      <c r="H15" t="str">
+        <v>HT-CONV-4455</v>
+      </c>
+      <c r="I15" t="str">
+        <v>2022-12-10</v>
+      </c>
+      <c r="J15" t="str">
+        <v>25000</v>
+      </c>
+      <c r="K15" t="str">
+        <v>2027-12-10</v>
+      </c>
+      <c r="L15" t="str">
+        <v>active</v>
+      </c>
+      <c r="M15" t="str">
+        <v>Main conveyor section for assembly line</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>TIG Welding Machine</v>
+      </c>
+      <c r="B16" t="str">
+        <v>AST-MACH-150</v>
+      </c>
+      <c r="C16" t="str">
+        <v>movable</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Machinery</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Workshop Area 3</v>
+      </c>
+      <c r="F16" t="str">
+        <v>Miller</v>
+      </c>
+      <c r="G16" t="str">
+        <v>Syncrowave 250</v>
+      </c>
+      <c r="H16" t="str">
+        <v>ML-WELD-5566</v>
+      </c>
+      <c r="I16" t="str">
+        <v>2024-02-25</v>
+      </c>
+      <c r="J16" t="str">
+        <v>7800</v>
+      </c>
+      <c r="K16" t="str">
+        <v>2026-02-25</v>
+      </c>
+      <c r="L16" t="str">
+        <v>active</v>
+      </c>
+      <c r="M16" t="str">
+        <v>Industrial TIG welder for aluminum and steel</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M16"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>